<commit_message>
market mapping 2026-09-29: XLSX consolide allege + decoupage en 3 parties pour envoi email
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PLUNgMZKuTHmV3LVeZzEnB
</commit_message>
<xml_diff>
--- a/outputs/humanup_market_mapping_2026-09-29.xlsx
+++ b/outputs/humanup_market_mapping_2026-09-29.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E211"/>
+  <dimension ref="A1:E108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -636,1231 +636,651 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>RAPPORT DE SYNTHESE</t>
+          <t>EXTRAIT DU RAPPORT DE SYNTHESE</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t># Rapport de synthèse — Market Mapping Humanup.io</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>**Date : 2026-09-29** (mardi)</t>
+          <t>Rapport complet : outputs/rapport_synthese_2026-09-29.md</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2. ⚠️ Alerte qualité du run — sourcing nominatif très dégradé</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>**20 contacts nominatifs sur 200 lignes (10 %)**, contre un objectif habituel bien supérieur.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>180 lignes portent le tag `CONTACT_NON_SOURCE` (nom, prénom et LinkedIn vides).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>## 1. Volumes par verticale</t>
+          <t>Deux causes techniques, aucune liée à la qualité des cibles :</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1. **Quota de recherche web saturé en début de run.** Le budget WebSearch est partagé entre tous</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>| Verticale | Destinataire | Lignes | Entreprises | Opportunités | Contacts sourcés | Taux |</t>
+          <t>les sous-agents (200 appels pour la session). Il a été consommé pendant la phase de détection</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>|---|---|---|---|---|---|---|</t>
+          <t>de récurrences et les 7 agents de sourcing lancés en parallèle, chacun n'ayant pu faire</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>| Finance / Comptabilité | Valentin Murcia | 40 | 20 | 14 JOB + 6 NEWS | 6 | 15 % |</t>
+          <t>qu'environ 14 recherches au lieu des 60-80 nécessaires. La phase de sourcing nominatif</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>| Hospitality / Restauration | Valentin Murcia | 40 | 20 | 14 JOB + 6 NEWS | 5 | 13 % |</t>
+          <t>(LinkedIn / Pappers, 3 essais par contact) n'a donc pas pu être menée sur la majorité des lignes.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>| Industrie | Alexis | 40 | 20 | 13 JOB + 7 NEWS | 1 | 3 % |</t>
+          <t>Les fichiers Industrie, Sales SaaS et Sales ont été complétés par un second passage (top-up)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>| Sales SaaS + portefeuille fonds | Louis | 40 | 20 | 13 JOB + 7 NEWS | 4 | 10 % |</t>
+          <t>une fois le quota reconstitué, ce qui a permis d'atteindre les 40 lignes partout.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>| Sales tous secteurs | Méroë Nguimbi | 40 | 20 | 14 JOB + 6 NEWS | 4 | 10 % |</t>
+          <t>2. **Egress proxy bloquant (403 EGRESS_BLOCKED)** sur l'ensemble des sources utiles :</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>| **TOTAL** | | **200** | **100** | **68 JOB + 32 NEWS** | **20** | **10 %** |</t>
+          <t>APEC, Indeed, Hellowork, France Travail, LinkedIn, Welcome to the Jungle, Pappers,</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Societe.com, Taleez, Usine Nouvelle, Journal des Palaces, L'Hôtellerie Restauration,</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Volume cible atteint sur les 5 verticales (40 lignes chacune).</t>
+          <t>Le Journal des Entreprises, LSA, Option Finance, DAF-Mag, et les sites corporate testés.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Tout le travail a donc reposé sur les snippets WebSearch.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>**Conséquences à connaître avant toute prospection :**</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>- **Dates d'annonces majoritairement `NC`** : la fenêtre stricte « publiée depuis moins de 7 jours »</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>## 2. ⚠️ Alerte qualité du run — sourcing nominatif très dégradé</t>
+          <t>n'est pas prouvée ligne par ligne. Les annonces sont confirmées *actives en septembre 2026*.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Seules quelques dates sont confirmées (POLYTECH 24/09, Sociabble 24/09, Ouest Conseils 19/09).</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>**20 contacts nominatifs sur 200 lignes (10 %)**, contre un objectif habituel bien supérieur.</t>
+          <t>- **Effectifs, CA et salaires majoritairement `NC`** — à confirmer avant appel.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>180 lignes portent le tag `CONTACT_NON_SOURCE` (nom, prénom et LinkedIn vides).</t>
+          <t>- Aucune donnée n'a été inventée : tout ce qui n'était pas confirmé est marqué `NC`, et aucun nom</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>de contact n'a été supposé. L'intégrité a été privilégiée sur le volume, conformément à la consigne.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Deux causes techniques, aucune liée à la qualité des cibles :</t>
+          <t>**Action recommandée :** relever le plafond de recherches web de la session</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>(`CLAUDE_CODE_MAX_WEB_SEARCHES_PER_SESSION`) et/ou séquencer les agents plutôt que de les lancer</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1. **Quota de recherche web saturé en début de run.** Le budget WebSearch est partagé entre tous</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   les sous-agents (200 appels pour la session). Il a été consommé pendant la phase de détection</t>
+          <t>tous les 7 en parallèle, pour restaurer le sourcing nominatif sur les prochains runs.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   de récurrences et les 7 agents de sourcing lancés en parallèle, chacun n'ayant pu faire</t>
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>4. Top 7 signaux business prioritaires</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">   qu'environ 14 recherches au lieu des 60-80 nécessaires. La phase de sourcing nominatif</t>
+          <t>1. **Maison Neyret (La Fouillouse, 42)** — 20 M€ investis, site Digitrace opérationnel en</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (LinkedIn / Pappers, 3 essais par contact) n'a donc pas pu être menée sur la majorité des lignes.</t>
+          <t>septembre 2026, **~100 postes au démarrage + 100 à venir**. Le plus gros volume de recrutement</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Les fichiers Industrie, Sales SaaS et Sales ont été complétés par un second passage (top-up)</t>
+          <t>industriel du jour.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">   une fois le quota reconstitué, ce qui a permis d'atteindre les 40 lignes partout.</t>
+          <t>2. **Kheops (Paris 12e)** — levée de **12 M€ le 21/09/2026** (Odyssée Venture + Isai + Elaia) avec</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2. **Egress proxy bloquant (403 EGRESS_BLOCKED)** sur l'ensemble des sources utiles :</t>
+          <t>**~30 recrutements annoncés dont des commerciaux**. Contact DG nominatif disponible</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">   APEC, Indeed, Hellowork, France Travail, LinkedIn, Welcome to the Jungle, Pappers,</t>
+          <t>(Caroline Poinsignon). Signal Sales SaaS le plus actionnable.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Societe.com, Taleez, Usine Nouvelle, Journal des Palaces, L'Hôtellerie Restauration,</t>
+          <t>3. **Biolevate (Paris)** — **Série A de 30 M€ le 22/09/2026** (RAISE France, Orange Ventures,</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Le Journal des Entreprises, LSA, Option Finance, DAF-Mag, et les sites corporate testés.</t>
+          <t>MSD GHI Fund, Station F, EQT Ventures). Montant le plus élevé de la fenêtre, phase de</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Tout le travail a donc reposé sur les snippets WebSearch.</t>
+          <t>structuration commerciale à venir.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr"/>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>4. **WeMa (Strasbourg, 430 sal, ~50 M€)** — LBO minoritaire : Kresk Développement entre à 20 %</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>**Conséquences à connaître avant toute prospection :**</t>
+          <t>(15-20 M€) + 105 M€ de dette Apera, stratégie de croissance externe à horizon 2030.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>- **Dates d'annonces majoritairement `NC`** : la fenêtre stricte « publiée depuis moins de 7 jours »</t>
+          <t>Double besoin finance + intégration.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">  n'est pas prouvée ligne par ligne. Les annonces sont confirmées *actives en septembre 2026*.</t>
+          <t>5. **DV GROUP (Hesdin, 62 — 350 sal, 50 M€)** — recrute **simultanément un RAF et un RAF adjoint**,</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Seules quelques dates sont confirmées (POLYTECH 24/09, Sociabble 24/09, Ouest Conseils 19/09).</t>
+          <t>sur fond de projets CSRD et de refonte ERP. Direction financière en pleine structuration :</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>- **Effectifs, CA et salaires majoritairement `NC`** — à confirmer avant appel.</t>
+          <t>cible idéale success-fee.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>- Aucune donnée n'a été inventée : tout ce qui n'était pas confirmé est marqué `NC`, et aucun nom</t>
+          <t>6. **Jacir / groupe Cofinair (Criquetot-sur-Longueville, 76)** — 25 M€, regroupement de 3 sites,</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">  de contact n'a été supposé. L'intégrité a été privilégiée sur le volume, conformément à la consigne.</t>
+          <t>160 salariés, CA 40 M€. Réorganisation industrielle génératrice de besoins production,</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr"/>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>maintenance et méthodes.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>**Action recommandée :** relever le plafond de recherches web de la session</t>
+          <t>7. **Groupe Anne-Sophie Pic** — ouverture d'**Anne-Sophie Pic Paris** à la Fondation Cartier le</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>(`CLAUDE_CODE_MAX_WEB_SEARCHES_PER_SESSION`) et/ou séquencer les agents plutôt que de les lancer</t>
+          <t>**18/09/2026** (date confirmée). Ouverture de table étoilée = besoins cuisine et salle immédiats.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>tous les 7 en parallèle, pour restaurer le sourcing nominatif sur les prochains runs.</t>
+          <t>**Autres signaux notables :** Wealthcome (15 M€, Breega + BlackFin, 24/09) · Kaiko (extension</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr"/>
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Série B à 110 M USD, 14/09) · Zeliq (extension seed 7 M€, 22/09) · DimoMaint (build-up triple,</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>fonds Keensight) · Groupe Fahrenheit (levée Bpifrance Tourisme 3 pour 2 hôtels 4\*) ·</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr"/>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Van Den Casteele (20 M€, +20 recrutements, 07/09) · Balsamo (siège Paris ouvert le 21/09) ·</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>## 3. Top régions / villes / secteurs</t>
+          <t>Charlott' (directrice commerciale promue DG le 03/09, pilotage force de vente VDI à repourvoir) ·</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr"/>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Groupe Charlois (DAF parti chez Agrial le 16/09, poste à repourvoir) ·</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Villes :** Paris (75) 40 lignes · Lyon (69) 12 · Nantes (44) 4 · Lille (59) 4 · Bordeaux (33) 4 ·</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Levallois-Perret (92) 2 · La Haie-Fouassière (44) 2 · Quimper (29) 2 · Reims (51) 2 · Toulon (83) 2 ·</t>
+          <t>Amarris Expertise Comptable (39 M€ levés, 8 cabinets intégrés).</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Strasbourg (67) 2. 10 lignes en localisation `NC`.</t>
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>5. Recurrences — entreprises déjà ciblées avec un signal frais (22 → 29/09/2026)</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr"/>
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>43 des 215 entreprises de la liste anti-doublons ont été re-vérifiées. **5 récurrences confirmées**</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Départements les plus représentés :** 75 (40) · 69 (18) · 59 (10) · 29 (8) · 83 (8) · 33 (8) ·</t>
+          <t>(élément concret ET daté dans la fenêtre 7 jours) :</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>44 (6) · 64 (6) · 62 (4) · 35 (4) · 03 (4) · 38 (4) · 34 (4) · 71 (4) · 57 (4).</t>
+          <t>- **Voyageurs du Monde** — OPA en cours + nouvelles offres. Projet de note en réponse à l'offre</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr"/>
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>publique d'Avantage déposé à l'AMF le 22/09 (180 €/action, sortie de cote visée), en parallèle de</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>**Équilibre géographique :** la consigne « privilégier les régions » est respectée sur Industrie</t>
+          <t>postes CDI publiés les 22, 23 et 28/09 (Paris, Lyon, Lausanne).</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>(La Fouillouse 42, Faulquemont 57, La Roche-sur-Yon 85, Eyrein 19, Bailleul 59, Criquetot 76,</t>
+          <t>- **Equativ** — acquisition de Kamino Retail annoncée le 26/09 pour étendre sa division retail media,</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Ligier 03, Cedrat 38) et sur Finance (Quimper, Reims, Toulon, Strasbourg, Nantes, Hesdin 62, Nice).</t>
+          <t>trois jours après son référencement comme partenaire technologique de ChatGPT Ads (23/09).</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Hospitality et Sales SaaS restent structurellement parisiens.</t>
+          <t>- **Stoïk** — ouverture le 23/09 de son premier programme partenaires MSP / infogéreurs /</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr"/>
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>intégrateurs : structuration d'un canal indirect, donc de besoins commerciaux.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>**Secteurs couverts :** expertise comptable indépendante et audit régional · direction financière</t>
+          <t>- **Groupe AGPM** — création annoncée le 25/09, avec KLESIA Mut', du fonds de dotation Joseph Kessel.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>de PME/ETI · hôtellerie indépendante et restauration étoilée · plasturgie, mécanique, composites,</t>
+          <t>Signal institutionnel plutôt que de recrutement.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>granulats, agroalimentaire, ENR, génie climatique · éditeurs SaaS B2B (BTP, RH, retail media,</t>
+          <t>- **PAREF Gestion** — renfort de l'équipe de développement annoncé à Patrimonia fin septembre :</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>legaltech, healthtech, fintech) · négoce technique, transport, télécom B2B, services au bâtiment.</t>
+          <t>arrivée d'Aodren Guillou comme directeur des réseaux de distribution, accompagné de deux</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr"/>
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>nouveaux collaborateurs.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>**Signaux proches mais hors fenêtre (utiles en relance) :** Ingeliance (plan de ~200 postes, offre</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr"/>
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>du 21/09, un jour trop tôt) · Shippingbo (acquisition de Baback le 17/09) · Hackuity (Série B</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>## 4. Top 7 signaux business prioritaires</t>
+          <t>19 M$ le 16/09) · Groupe Okwind (cession de Purecontrol le 16/09, DAF nommé le 07/09) ·</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr"/>
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Cité Marine (40 M€ d'investissement Morbihan, ~38 offres actives, date non confirmée) ·</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>1. **Maison Neyret (La Fouillouse, 42)** — 20 M€ investis, site Digitrace opérationnel en</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   septembre 2026, **~100 postes au démarrage + 100 à venir**. Le plus gros volume de recrutement</t>
+          <t>Maisons Pariente (nouvelle DRH, ouverture Saint Roch Courchevel en décembre 2026).</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   industriel du jour.</t>
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>7. Dédoublonnage Sales Méroë ↔ Louis</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2. **Kheops (Paris 12e)** — levée de **12 M€ le 21/09/2026** (Odyssée Venture + Isai + Elaia) avec</t>
+          <t>Dédoublonnage exécuté sur la colonne `entreprise` (normalisation casse et espaces) :</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">   **~30 recrutements annoncés dont des commerciaux**. Contact DG nominatif disponible</t>
+          <t>**0 entreprise retirée**, le fichier de Méroë conserve ses **40 lignes / 20 entreprises**.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (Caroline Poinsignon). Signal Sales SaaS le plus actionnable.</t>
+          <t>Les deux agents Sales ont travaillé sur des périmètres disjoints — Louis sur les éditeurs SaaS et</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>3. **Biolevate (Paris)** — **Série A de 30 M€ le 22/09/2026** (RAISE France, Orange Ventures,</t>
+          <t>tech B2B, Méroë sur l'industrie, le négoce technique, le transport, les services au bâtiment,</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">   MSD GHI Fund, Station F, EQT Ventures). Montant le plus élevé de la fenêtre, phase de</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   structuration commerciale à venir.</t>
+          <t>la télécom B2B, les ENR et l'agroalimentaire — ce qui a évité tout chevauchement en amont.</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>4. **WeMa (Strasbourg, 430 sal, ~50 M€)** — LBO minoritaire : Kresk Développement entre à 20 %</t>
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>8. Points de vigilance à valider avant appel</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (15-20 M€) + 105 M€ de dette Apera, stratégie de croissance externe à horizon 2030.</t>
+          <t>- **CAP INGELEC** (Industrie) — effectif groupe non vérifié, à confirmer sous 2000 salariés.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Double besoin finance + intégration.</t>
+          <t>- **SEFI** (Sales) — 45 agences annoncées, effectif groupe à confirmer.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>5. **DV GROUP (Hesdin, 62 — 350 sal, 50 M€)** — recrute **simultanément un RAF et un RAF adjoint**,</t>
+          <t>- **Groupe Galopin** (Sales) — effectif groupe non confirmé.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">   sur fond de projets CSRD et de refonte ERP. Direction financière en pleine structuration :</t>
+          <t>- **Groupe Charlois** (Finance) — localisation et effectif en `NC`.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">   cible idéale success-fee.</t>
+          <t>- **Obat** (Sales SaaS) — levée de 12 M€ confirmée mais **date non confirmée**, potentiellement</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>6. **Jacir / groupe Cofinair (Criquetot-sur-Longueville, 76)** — 25 M€, regroupement de 3 sites,</t>
+          <t>antérieure à 30 jours : à vérifier avant de l'utiliser comme signal news.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">   160 salariés, CA 40 M€. Réorganisation industrielle génératrice de besoins production,</t>
+          <t>- **Ouest Conseils** (Finance) — annonce datée du 19/09, légèrement hors fenêtre 7 jours.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t xml:space="preserve">   maintenance et méthodes.</t>
+          <t>- **Groupe Daniel** (Sales) — annonce du 29/07, hors fenêtre 7 jours, conservée pour la qualité</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>7. **Groupe Anne-Sophie Pic** — ouverture d'**Anne-Sophie Pic Paris** à la Fondation Cartier le</t>
+          <t>du signal (Directeur Commercial au CODIR pilotant ~15 commerciaux).</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">   **18/09/2026** (date confirmée). Ouverture de table étoilée = besoins cuisine et salle immédiats.</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>**Autres signaux notables :** Wealthcome (15 M€, Breega + BlackFin, 24/09) · Kaiko (extension</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>Série B à 110 M USD, 14/09) · Zeliq (extension seed 7 M€, 22/09) · DimoMaint (build-up triple,</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>fonds Keensight) · Groupe Fahrenheit (levée Bpifrance Tourisme 3 pour 2 hôtels 4\*) ·</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>Van Den Casteele (20 M€, +20 recrutements, 07/09) · Balsamo (siège Paris ouvert le 21/09) ·</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>Charlott' (directrice commerciale promue DG le 03/09, pilotage force de vente VDI à repourvoir) ·</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>Groupe Charlois (DAF parti chez Agrial le 16/09, poste à repourvoir) ·</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Amarris Expertise Comptable (39 M€ levés, 8 cabinets intégrés).</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr"/>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr"/>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>## 5. Recurrences — entreprises déjà ciblées avec un signal frais (22 → 29/09/2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr"/>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>43 des 215 entreprises de la liste anti-doublons ont été re-vérifiées. **5 récurrences confirmées**</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>(élément concret ET daté dans la fenêtre 7 jours) :</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr"/>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>- **Voyageurs du Monde** — OPA en cours + nouvelles offres. Projet de note en réponse à l'offre</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  publique d'Avantage déposé à l'AMF le 22/09 (180 €/action, sortie de cote visée), en parallèle de</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  postes CDI publiés les 22, 23 et 28/09 (Paris, Lyon, Lausanne).</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>- **Equativ** — acquisition de Kamino Retail annoncée le 26/09 pour étendre sa division retail media,</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  trois jours après son référencement comme partenaire technologique de ChatGPT Ads (23/09).</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>- **Stoïk** — ouverture le 23/09 de son premier programme partenaires MSP / infogéreurs /</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  intégrateurs : structuration d'un canal indirect, donc de besoins commerciaux.</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>- **Groupe AGPM** — création annoncée le 25/09, avec KLESIA Mut', du fonds de dotation Joseph Kessel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Signal institutionnel plutôt que de recrutement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>- **PAREF Gestion** — renfort de l'équipe de développement annoncé à Patrimonia fin septembre :</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  arrivée d'Aodren Guillou comme directeur des réseaux de distribution, accompagné de deux</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  nouveaux collaborateurs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr"/>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>**Signaux proches mais hors fenêtre (utiles en relance) :** Ingeliance (plan de ~200 postes, offre</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>du 21/09, un jour trop tôt) · Shippingbo (acquisition de Baback le 17/09) · Hackuity (Série B</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>19 M$ le 16/09) · Groupe Okwind (cession de Purecontrol le 16/09, DAF nommé le 07/09) ·</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>Cité Marine (40 M€ d'investissement Morbihan, ~38 offres actives, date non confirmée) ·</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>Maisons Pariente (nouvelle DRH, ouverture Saint Roch Courchevel en décembre 2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr"/>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr"/>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>## 6. Filtres appliqués</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr"/>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>**Anti-doublons 14 jours :** 215 entreprises issues de 32 fichiers CSV (15 → 25/09) exclues de la</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>recherche. Contrôle programmatique dans chaque agent : **0 collision** sur les 5 fichiers livrés.</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr"/>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>**Plafond effectif groupe &lt; 2000 salariés :** entreprises écartées pendant la recherche —</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>Suez, Fives, Covéa, Crédit Agricole, Société Générale, Chausson Matériaux, Knauf, Amphenol,</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>ID Logistics, Record/Assa Abloy, Actemium/Vinci, Massilly, Bertin/CNIM, Pigeon Granulats, Symrise,</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>Staub/Zwilling, PPG, Cooperl, Atlantic, Arabelle Solutions, Verisure, Sector Alarm, Timac Agro</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>(Roullier), Cultura, CHEP, Primagaz, MAN FS, Finimetal (Purmo ~7000 sal), Groupe Berto (~3000 sal),</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>Larivère, MasterGrid, CHG-Meridian, Schmidt Groupe, Ponticelli, Point.P, Eureden, Laboratoires UMA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr"/>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>**Groupes hôteliers exclus par principe :** Accor, Marriott, Hilton, IHG, Hyatt, Rosewood,</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>Four Seasons, Mandarin Oriental. Écartés à ce titre ou pour doublon : Le Bristol (Oetker),</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>Hôtel Sax (Hilton), Château de Cîteaux (Fontenille Collection), Summer Hotels, Maisons Pariente,</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>Domaine Les Crayères.</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr"/>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>**Liste noire respectée :** aucun Big 4, next tier, réseau d'expertise comptable, scale-up</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>surmédiatisée ni CAC 40 dans les livrables. Sales SaaS : Oodrive, Doctrine, iAdvize, Modjo, Dastra,</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>Siteflow, Tenacy, Zei écartés (ex-FT120 ou déjà ciblés).</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr"/>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>**Cabinets masquant l'employeur final écartés :** L'Heureux Talent, Genesis RH, Talenteeds, Projex,</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>Imperium, Tryon, SwiftTalent, Vidal Associates, Fed Finance, Michael Page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr"/>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>**Exclusion alternance / stage :** appliquée sur tous les intitulés retenus.</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr"/>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr"/>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>## 7. Dédoublonnage Sales Méroë ↔ Louis</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr"/>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>Dédoublonnage exécuté sur la colonne `entreprise` (normalisation casse et espaces) :</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>**0 entreprise retirée**, le fichier de Méroë conserve ses **40 lignes / 20 entreprises**.</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>Les deux agents Sales ont travaillé sur des périmètres disjoints — Louis sur les éditeurs SaaS et</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>tech B2B, Méroë sur l'industrie, le négoce technique, le transport, les services au bâtiment,</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>la télécom B2B, les ENR et l'agroalimentaire — ce qui a évité tout chevauchement en amont.</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr"/>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr"/>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>## 8. Points de vigilance à valider avant appel</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr"/>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>- **CAP INGELEC** (Industrie) — effectif groupe non vérifié, à confirmer sous 2000 salariés.</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>- **SEFI** (Sales) — 45 agences annoncées, effectif groupe à confirmer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>- **Groupe Galopin** (Sales) — effectif groupe non confirmé.</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>- **Groupe Charlois** (Finance) — localisation et effectif en `NC`.</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>- **Obat** (Sales SaaS) — levée de 12 M€ confirmée mais **date non confirmée**, potentiellement</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  antérieure à 30 jours : à vérifier avant de l'utiliser comme signal news.</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>- **Ouest Conseils** (Finance) — annonce datée du 19/09, légèrement hors fenêtre 7 jours.</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>- **Groupe Daniel** (Sales) — annonce du 29/07, hors fenêtre 7 jours, conservée pour la qualité</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  du signal (Directeur Commercial au CODIR pilotant ~15 commerciaux).</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
           <t>- **CENISIS LILLE** (Finance) — 20-49 salariés, CA 3,0 M€ : retenue au titre de la tolérance 5-50 sal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr"/>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr"/>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>## 9. Fichiers livrés</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr"/>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>| Fichier | Destinataire |</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>|---|---|</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>| `outputs/finance_2026-09-29.csv` | Valentin Murcia |</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>| `outputs/hospitality_2026-09-29.csv` | Valentin Murcia |</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>| `outputs/industrie_2026-09-29.csv` | Alexis |</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>| `outputs/sales_saas_2026-09-29.csv` | Louis |</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>| `outputs/sales_2026-09-29.csv` | Méroë Nguimbi |</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>| `outputs/humanup_market_mapping_2026-09-29.xlsx` | Méroë Nguimbi (consolidé 6 onglets) |</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>| `outputs/rapport_synthese_2026-09-29.md` | Méroë Nguimbi |</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr"/>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>Fichiers intermédiaires Finance conservés : `_fin_a_`, `_fin_b_`, `_fin_c_2026-09-29.csv`.</t>
         </is>
       </c>
     </row>

</xml_diff>